<commit_message>
Add binary to ternary figure
</commit_message>
<xml_diff>
--- a/20240512_SA_binary/output/system_analysis/system_analysis_files.xlsx
+++ b/20240512_SA_binary/output/system_analysis/system_analysis_files.xlsx
@@ -31,6 +31,12 @@
     <t>In-In</t>
   </si>
   <si>
+    <t>451606_bi</t>
+  </si>
+  <si>
+    <t>451623_bi</t>
+  </si>
+  <si>
     <t>450249_bi</t>
   </si>
   <si>
@@ -43,25 +49,19 @@
     <t>457677_bi</t>
   </si>
   <si>
-    <t>451606_bi</t>
-  </si>
-  <si>
     <t>1538436_bi</t>
   </si>
   <si>
-    <t>451623_bi</t>
+    <t>U3Si2</t>
+  </si>
+  <si>
+    <t>Mg2Cu</t>
   </si>
   <si>
     <t>IrIn3</t>
   </si>
   <si>
-    <t>U3Si2</t>
-  </si>
-  <si>
     <t>RuIn3</t>
-  </si>
-  <si>
-    <t>Mg2Cu</t>
   </si>
   <si>
     <t>All files</t>
@@ -470,7 +470,7 @@
         <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -487,7 +487,7 @@
         <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -504,7 +504,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -521,7 +521,7 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6">
         <v>0</v>

</xml_diff>